<commit_message>
test: verify every hourly workbook filter result
</commit_message>
<xml_diff>
--- a/outputs/portfolio-2026-10-17/Dockside_Analysis.xlsx
+++ b/outputs/portfolio-2026-10-17/Dockside_Analysis.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8b0462e17644426c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stations" sheetId="2" r:id="Rbd8d2de1296245ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily coverage" sheetId="3" r:id="Rbc1af07b8d30439e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Time patterns" sheetId="4" r:id="R1162328e947b4e6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nearby alternatives" sheetId="5" r:id="R612824cca86c4100"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source QA" sheetId="6" r:id="R202e52df451e40c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R15c171ef703a4bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf69e7fa2d1184261"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stations" sheetId="2" r:id="R12c495f7ec05401e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily coverage" sheetId="3" r:id="R0864c7f6611b458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Time patterns" sheetId="4" r:id="Rb8acb12526724ae0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nearby alternatives" sheetId="5" r:id="Rd39d3955547d40ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source QA" sheetId="6" r:id="Racae670ec6064b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="7" r:id="R04ab0c2a09144048"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="StationIDs">'Stations'!B7:B1081</x:definedName>
@@ -523,7 +523,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R228e068208744dbf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc311f3a6d7974e6d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -558,7 +558,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rac8e58f246d54e8e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R932ae52c8eed4c3e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2048,7 +2048,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R760cea3df37f498e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dd34c32d7c24cd9"/>
 </x:worksheet>
 </file>
 
@@ -46451,7 +46451,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f692f559c064bcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re58b5e573a3e49f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -48148,7 +48148,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7feb14fe12b34c5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R496a5b427e394137"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -50106,9 +50106,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76ac28c287a147a3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf52f365336ea4300"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d162d5556b74648"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a827a7dd7004294"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -51124,7 +51124,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4462ee521bb1413c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0081f9e57be41e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52175,10 +52175,10 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re687f2c1727a45ca"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b50abc28a994edc"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re93743cf7c9a486a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f0c15665dfe41bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb477d4223a2d4e67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84e7d63bef5b4ae3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd6eb99564224a3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e79588efb1c4f30"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>